<commit_message>
ADIB: the sanctioned beta written where a gate outside the study can read it
</commit_message>
<xml_diff>
--- a/engine/swdy_study/SWDY_Valuation_Model_09092026_public.xlsx
+++ b/engine/swdy_study/SWDY_Valuation_Model_09092026_public.xlsx
@@ -2560,19 +2560,19 @@
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>48.0507329597046</v>
+        <v>51.75154484595317</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>49.70216467416559</v>
+        <v>53.58598972095123</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>51.61377072512412</v>
+        <v>55.71660640416448</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>53.8702170590966</v>
+        <v>58.23977514128349</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>56.59737534073271</v>
+        <v>61.29878307978106</v>
       </c>
     </row>
     <row r="7">
@@ -2582,19 +2582,19 @@
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>43.38965839771769</v>
+        <v>46.92330884452585</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>44.58953433723649</v>
+        <v>48.27673925934022</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>45.94722493645097</v>
+        <v>49.81551773527278</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>47.50906063258347</v>
+        <v>51.59405782760725</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>49.34147433400587</v>
+        <v>53.69038277439329</v>
       </c>
     </row>
     <row r="8">
@@ -2604,19 +2604,19 @@
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>39.39440569105454</v>
+        <v>42.78567612194627</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>40.25970494315277</v>
+        <v>43.7814301475257</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>41.21632469837968</v>
+        <v>44.89000036914447</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>42.28868469751839</v>
+        <v>46.14155462610511</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>43.51076338157681</v>
+        <v>47.57806945522615</v>
       </c>
     </row>
     <row r="9">
@@ -2626,19 +2626,19 @@
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>35.93336189108932</v>
+        <v>39.20208987342894</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>36.54718264711511</v>
+        <v>39.92793436920949</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>37.20843070440687</v>
+        <v>40.71828410658065</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>37.92875051852907</v>
+        <v>41.58897655466522</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>38.72393829011554</v>
+        <v>42.56149591582977</v>
       </c>
     </row>
     <row r="10">
@@ -2648,19 +2648,19 @@
         </is>
       </c>
       <c r="B10" s="7" t="n">
-        <v>32.90738826514143</v>
+        <v>36.06968942362016</v>
       </c>
       <c r="C10" s="7" t="n">
-        <v>33.32998437664673</v>
+        <v>36.58938119058816</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>33.77073485461407</v>
+        <v>37.14100170621704</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>34.23375980649833</v>
+        <v>37.73179715426411</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>34.72452811024157</v>
+        <v>38.3713858505013</v>
       </c>
     </row>
     <row r="12">
@@ -2705,19 +2705,19 @@
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>60.17049350743897</v>
+        <v>65.07928889866324</v>
       </c>
       <c r="C14" s="7" t="n">
-        <v>58.35223880309312</v>
+        <v>63.15563431199472</v>
       </c>
       <c r="D14" s="7" t="n">
-        <v>56.59737534073271</v>
+        <v>61.29878307978106</v>
       </c>
       <c r="E14" s="7" t="n">
-        <v>54.90314327729129</v>
+        <v>59.50583189191774</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>53.26692765802384</v>
+        <v>57.77402971679158</v>
       </c>
     </row>
     <row r="15">
@@ -2727,19 +2727,19 @@
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>52.50650406475745</v>
+        <v>57.04303387246198</v>
       </c>
       <c r="C15" s="7" t="n">
-        <v>50.89597043113798</v>
+        <v>55.3371612118944</v>
       </c>
       <c r="D15" s="7" t="n">
-        <v>49.34147433400587</v>
+        <v>53.69038277439329</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>47.84057999237388</v>
+        <v>52.1001349503897</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>46.39097933936378</v>
+        <v>50.56398840677389</v>
       </c>
     </row>
     <row r="16">
@@ -2749,19 +2749,19 @@
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>46.34801613119999</v>
+        <v>50.58716923736989</v>
       </c>
       <c r="C16" s="7" t="n">
-        <v>44.90432296618077</v>
+        <v>49.05616591921513</v>
       </c>
       <c r="D16" s="7" t="n">
-        <v>43.51076338157681</v>
+        <v>47.57806945522615</v>
       </c>
       <c r="E16" s="7" t="n">
-        <v>42.16516167246377</v>
+        <v>46.15058877372767</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>40.86545606942517</v>
+        <v>44.77155264158418</v>
       </c>
     </row>
     <row r="17">
@@ -2771,19 +2771,19 @@
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>41.29223410819131</v>
+        <v>45.28878322593069</v>
       </c>
       <c r="C17" s="7" t="n">
-        <v>39.98544052927011</v>
+        <v>43.90122265074462</v>
       </c>
       <c r="D17" s="7" t="n">
-        <v>38.72393829011554</v>
+        <v>42.56149591582977</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>37.50576490546236</v>
+        <v>41.26753530950558</v>
       </c>
       <c r="F17" s="7" t="n">
-        <v>36.3290605333606</v>
+        <v>40.01738113023824</v>
       </c>
     </row>
     <row r="18">
@@ -2793,19 +2793,19 @@
         </is>
       </c>
       <c r="B18" s="7" t="n">
-        <v>37.06823178367044</v>
+        <v>40.86342268675902</v>
       </c>
       <c r="C18" s="7" t="n">
-        <v>35.87575503510264</v>
+        <v>39.5956036862078</v>
       </c>
       <c r="D18" s="7" t="n">
-        <v>34.72452811024157</v>
+        <v>38.3713858505013</v>
       </c>
       <c r="E18" s="7" t="n">
-        <v>33.61276640826723</v>
+        <v>37.18888774615379</v>
       </c>
       <c r="F18" s="7" t="n">
-        <v>32.53877855437916</v>
+        <v>36.04632608893751</v>
       </c>
     </row>
     <row r="20">
@@ -2840,19 +2840,19 @@
         </is>
       </c>
       <c r="B22" s="7" t="n">
-        <v>82.89233633171949</v>
+        <v>88.94087384303364</v>
       </c>
       <c r="C22" s="7" t="n">
-        <v>65.99151475122238</v>
+        <v>71.1924064433187</v>
       </c>
       <c r="D22" s="7" t="n">
-        <v>46.59451573941893</v>
+        <v>50.81803765134803</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>43.50709365611225</v>
+        <v>47.57421363061231</v>
       </c>
       <c r="F22" s="7" t="n">
-        <v>40.69096331071587</v>
+        <v>44.61511461402405</v>
       </c>
       <c r="H22" s="16">
         <f>MAX(B22:F22)-MIN(B22:F22)</f>
@@ -2866,19 +2866,19 @@
         </is>
       </c>
       <c r="B23" s="7" t="n">
-        <v>42.07500523515485</v>
+        <v>47.57806945522615</v>
       </c>
       <c r="C23" s="7" t="n">
-        <v>43.51076338157681</v>
+        <v>47.57806945522615</v>
       </c>
       <c r="D23" s="7" t="n">
-        <v>46.38227967442072</v>
+        <v>47.57806945522615</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>49.97167504047564</v>
+        <v>47.57806945522615</v>
       </c>
       <c r="F23" s="7" t="n">
-        <v>53.56107040653055</v>
+        <v>47.57806945522615</v>
       </c>
       <c r="H23" s="16">
         <f>MAX(B23:F23)-MIN(B23:F23)</f>
@@ -2892,19 +2892,19 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>23.17689166022818</v>
+        <v>26.73474268688304</v>
       </c>
       <c r="C24" s="7" t="n">
-        <v>33.3438275209025</v>
+        <v>37.15640607105463</v>
       </c>
       <c r="D24" s="7" t="n">
-        <v>43.51076338157681</v>
+        <v>47.57806945522615</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>53.67769924225113</v>
+        <v>57.99973283939774</v>
       </c>
       <c r="F24" s="7" t="n">
-        <v>63.84463510292543</v>
+        <v>68.42139622356929</v>
       </c>
       <c r="H24" s="16">
         <f>MAX(B24:F24)-MIN(B24:F24)</f>
@@ -2918,19 +2918,19 @@
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>41.3571261619439</v>
+        <v>47.57806945522615</v>
       </c>
       <c r="C25" s="7" t="n">
-        <v>42.43394477176034</v>
+        <v>47.57806945522615</v>
       </c>
       <c r="D25" s="7" t="n">
-        <v>43.51076338157681</v>
+        <v>47.57806945522615</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>44.58758199139326</v>
+        <v>47.57806945522615</v>
       </c>
       <c r="F25" s="7" t="n">
-        <v>45.66440060120974</v>
+        <v>47.57806945522615</v>
       </c>
       <c r="H25" s="16">
         <f>MAX(B25:F25)-MIN(B25:F25)</f>
@@ -2944,19 +2944,19 @@
         </is>
       </c>
       <c r="B26" s="7" t="n">
-        <v>50.27171997464177</v>
+        <v>54.35297381891678</v>
       </c>
       <c r="C26" s="7" t="n">
-        <v>46.77467346098749</v>
+        <v>50.84871294114577</v>
       </c>
       <c r="D26" s="7" t="n">
-        <v>43.51076338157681</v>
+        <v>47.57806945522615</v>
       </c>
       <c r="E26" s="7" t="n">
-        <v>39.7805804336789</v>
+        <v>43.84019118560374</v>
       </c>
       <c r="F26" s="7" t="n">
-        <v>36.28353392002459</v>
+        <v>40.33593030783275</v>
       </c>
       <c r="H26" s="16">
         <f>MAX(B26:F26)-MIN(B26:F26)</f>
@@ -2966,23 +2966,23 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>Terminal return on invested capital  (15.0% / 18.0% / 20.1% / 26.0% / 30.0%)</t>
+          <t>Terminal return on invested capital  (15.0% / 18.0% / 20.8% / 26.0% / 30.0%)</t>
         </is>
       </c>
       <c r="B27" s="7" t="n">
-        <v>40.98127111072365</v>
+        <v>44.5245675843202</v>
       </c>
       <c r="C27" s="7" t="n">
-        <v>46.71205527626227</v>
+        <v>50.44728335978145</v>
       </c>
       <c r="D27" s="7" t="n">
-        <v>49.7075887045515</v>
+        <v>54.475229952078</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>55.52864630016783</v>
+        <v>59.55915378356799</v>
       </c>
       <c r="F27" s="7" t="n">
-        <v>58.17362360733951</v>
+        <v>62.29271491070394</v>
       </c>
       <c r="H27" s="16">
         <f>MAX(B27:F27)-MIN(B27:F27)</f>
@@ -2996,19 +2996,19 @@
         </is>
       </c>
       <c r="B28" s="7" t="n">
-        <v>39.39440569105454</v>
+        <v>42.78567612194627</v>
       </c>
       <c r="C28" s="7" t="n">
-        <v>40.25970494315277</v>
+        <v>43.7814301475257</v>
       </c>
       <c r="D28" s="7" t="n">
-        <v>41.21632469837968</v>
+        <v>44.89000036914447</v>
       </c>
       <c r="E28" s="7" t="n">
-        <v>42.28868469751839</v>
+        <v>46.14155462610511</v>
       </c>
       <c r="F28" s="7" t="n">
-        <v>43.51076338157681</v>
+        <v>47.57806945522615</v>
       </c>
       <c r="H28" s="16">
         <f>MAX(B28:F28)-MIN(B28:F28)</f>
@@ -3710,7 +3710,7 @@
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>Terminal growth reconciliation: actual NOPAT compound growth FY2023–FY2025 was 26.9%; the implied growth from stable years only (FY2024 excluded as a debt-funded capacity burst) is 7.6%; the adopted terminal growth is 7.0%, below the blended nominal ceiling of 11.1%.</t>
+          <t>Terminal growth reconciliation: actual NOPAT compound growth FY2023–FY2025 was 26.9%; the implied growth from stable years only (FY2024 excluded as a debt-funded capacity burst) is 7.6%; the adopted terminal growth is 7.0%, below the blended nominal ceiling of 11.2%.</t>
         </is>
       </c>
     </row>
@@ -4015,14 +4015,14 @@
         </is>
       </c>
       <c r="B5" s="7" t="n">
-        <v>16.18162005664932</v>
+        <v>18.93534675964298</v>
       </c>
       <c r="C5" s="8">
         <f>DCF!C62</f>
         <v/>
       </c>
       <c r="D5" s="7" t="n">
-        <v>83.79876343050132</v>
+        <v>85.99664201115992</v>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
@@ -4428,7 +4428,7 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>16.18162005664932</v>
+        <v>18.93534675964298</v>
       </c>
     </row>
     <row r="7">
@@ -4443,7 +4443,7 @@
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>83.79876343050132</v>
+        <v>85.99664201115992</v>
       </c>
     </row>
     <row r="8">
@@ -4520,7 +4520,7 @@
         </is>
       </c>
       <c r="C15" s="21" t="n">
-        <v>0.5254856747391311</v>
+        <v>0.5121665673676995</v>
       </c>
     </row>
     <row r="16">
@@ -4553,7 +4553,7 @@
         </is>
       </c>
       <c r="C18" s="7" t="n">
-        <v>57.86095793273499</v>
+        <v>60.92524917987439</v>
       </c>
     </row>
     <row r="19">
@@ -4613,13 +4613,13 @@
         </is>
       </c>
       <c r="C23" s="7" t="n">
-        <v>153.052652198775</v>
+        <v>157.9819478660362</v>
       </c>
       <c r="D23" s="7" t="n">
-        <v>112.2887963569921</v>
+        <v>115.9209089539214</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>193.8165080405579</v>
+        <v>200.0429867781509</v>
       </c>
     </row>
     <row r="24">
@@ -4634,13 +4634,13 @@
         </is>
       </c>
       <c r="C24" s="7" t="n">
-        <v>65.48394099946414</v>
+        <v>64.40329970107479</v>
       </c>
       <c r="D24" s="7" t="n">
-        <v>34.12367903228015</v>
+        <v>33.54633805623964</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>59.75270243066323</v>
+        <v>58.7640416846734</v>
       </c>
     </row>
     <row r="25">
@@ -4655,13 +4655,13 @@
         </is>
       </c>
       <c r="C25" s="7" t="n">
-        <v>45.28950840983638</v>
+        <v>50.06967725437205</v>
       </c>
       <c r="D25" s="7" t="n">
-        <v>42.22747080432825</v>
+        <v>44.9626128412424</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>57.86095793273499</v>
+        <v>60.92524917987439</v>
       </c>
     </row>
     <row r="26">
@@ -4816,7 +4816,7 @@
         </is>
       </c>
       <c r="C9" s="25" t="n">
-        <v>49.5</v>
+        <v>47.69</v>
       </c>
     </row>
     <row r="11">
@@ -5076,19 +5076,19 @@
         </is>
       </c>
       <c r="B26" s="21" t="n">
-        <v>0.044</v>
+        <v>0.03574226695658529</v>
       </c>
       <c r="C26" s="21" t="n">
-        <v>0.04</v>
+        <v>0.03574226695658529</v>
       </c>
       <c r="D26" s="21" t="n">
-        <v>0.036</v>
+        <v>0.03574226695658529</v>
       </c>
       <c r="E26" s="21" t="n">
-        <v>0.033</v>
+        <v>0.03574226695658529</v>
       </c>
       <c r="F26" s="21" t="n">
-        <v>0.031</v>
+        <v>0.03574226695658529</v>
       </c>
     </row>
     <row r="27">
@@ -5402,7 +5402,7 @@
         </is>
       </c>
       <c r="C58" s="24" t="n">
-        <v>110489.8413121987</v>
+        <v>110761.3616516914</v>
       </c>
     </row>
     <row r="59">
@@ -5852,19 +5852,19 @@
         <v>0.134899552356732</v>
       </c>
       <c r="E5" s="24" t="n">
-        <v>221541.3228857327</v>
+        <v>203416.1993989137</v>
       </c>
       <c r="F5" s="24" t="n">
-        <v>252428.7347156312</v>
+        <v>231776.5966461021</v>
       </c>
       <c r="G5" s="24" t="n">
-        <v>276853.5521024677</v>
+        <v>254203.1284512111</v>
       </c>
       <c r="H5" s="24" t="n">
-        <v>302516.6726712704</v>
+        <v>277766.6532276451</v>
       </c>
       <c r="I5" s="24" t="n">
-        <v>329470.412277309</v>
+        <v>302515.206675059</v>
       </c>
     </row>
     <row r="6">
@@ -5884,19 +5884,19 @@
         <v>0.06452269254829619</v>
       </c>
       <c r="E6" s="24" t="n">
-        <v>107331.08926904</v>
+        <v>115920.4463847608</v>
       </c>
       <c r="F6" s="24" t="n">
-        <v>122357.4417667056</v>
+        <v>132149.3088786273</v>
       </c>
       <c r="G6" s="24" t="n">
-        <v>135816.7603610432</v>
+        <v>146685.7328552763</v>
       </c>
       <c r="H6" s="24" t="n">
-        <v>148040.2687935371</v>
+        <v>159887.4488122512</v>
       </c>
       <c r="I6" s="24" t="n">
-        <v>159883.4902970201</v>
+        <v>172678.4447172313</v>
       </c>
     </row>
     <row r="7">
@@ -5916,19 +5916,19 @@
         <v>0.2217300370961013</v>
       </c>
       <c r="E7" s="24" t="n">
-        <v>41157.1221036</v>
+        <v>50857.09276164287</v>
       </c>
       <c r="F7" s="24" t="n">
-        <v>47742.261640176</v>
+        <v>58994.22760350573</v>
       </c>
       <c r="G7" s="24" t="n">
-        <v>53948.75565339887</v>
+        <v>66663.47719196147</v>
       </c>
       <c r="H7" s="24" t="n">
-        <v>59883.11877527275</v>
+        <v>73996.45968307724</v>
       </c>
       <c r="I7" s="24" t="n">
-        <v>65871.43065280003</v>
+        <v>81396.10565138496</v>
       </c>
     </row>
     <row r="8">
@@ -6006,19 +6006,19 @@
         </is>
       </c>
       <c r="B11" s="24" t="n">
-        <v>25331.25640007756</v>
+        <v>23258.81165547119</v>
       </c>
       <c r="C11" s="24" t="n">
-        <v>28862.95395611998</v>
+        <v>26501.56783711195</v>
       </c>
       <c r="D11" s="24" t="n">
-        <v>31655.71200094826</v>
+        <v>29065.83991023992</v>
       </c>
       <c r="E11" s="24" t="n">
-        <v>34590.05886990573</v>
+        <v>31760.11689670217</v>
       </c>
       <c r="F11" s="24" t="n">
-        <v>37671.97641019979</v>
+        <v>34589.89124643293</v>
       </c>
     </row>
     <row r="12">
@@ -6028,19 +6028,19 @@
         </is>
       </c>
       <c r="B12" s="24" t="n">
-        <v>9645.952323697893</v>
+        <v>10417.88643704483</v>
       </c>
       <c r="C12" s="24" t="n">
-        <v>10996.3856490156</v>
+        <v>11876.39053823111</v>
       </c>
       <c r="D12" s="24" t="n">
-        <v>12205.98807040732</v>
+        <v>13182.79349743654</v>
       </c>
       <c r="E12" s="24" t="n">
-        <v>13304.52699674398</v>
+        <v>14369.24491220583</v>
       </c>
       <c r="F12" s="24" t="n">
-        <v>14368.8891564835</v>
+        <v>15518.7845051823</v>
       </c>
     </row>
     <row r="13">
@@ -6050,19 +6050,19 @@
         </is>
       </c>
       <c r="B13" s="24" t="n">
-        <v>9722.176540434495</v>
+        <v>12013.51330924804</v>
       </c>
       <c r="C13" s="24" t="n">
-        <v>11277.72478690401</v>
+        <v>13935.67543872773</v>
       </c>
       <c r="D13" s="24" t="n">
-        <v>12743.82900920153</v>
+        <v>15747.31324576233</v>
       </c>
       <c r="E13" s="24" t="n">
-        <v>14145.6502002137</v>
+        <v>17479.51770279619</v>
       </c>
       <c r="F13" s="24" t="n">
-        <v>15560.21522023508</v>
+        <v>19227.46947307581</v>
       </c>
     </row>
     <row r="14">

</xml_diff>

<commit_message>
SWDY artefacts rebuilt on the corrected terminal
Study, workbook and bibliography regenerated after the terminal risk-free was derived
from the house macro path. recalc reports every formula cell reproducing the model.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017RcjXG4ETjADcoFJf123yY
</commit_message>
<xml_diff>
--- a/engine/swdy_study/SWDY_Valuation_Model_09092026_public.xlsx
+++ b/engine/swdy_study/SWDY_Valuation_Model_09092026_public.xlsx
@@ -808,7 +808,7 @@
     <row r="42">
       <c r="A42" s="3" t="inlineStr">
         <is>
-          <t>28.8% -&gt; 17.2% on the same easing calendar as the interest forecast; the terminal value is</t>
+          <t>28.8% -&gt; 18.9% on the same easing calendar as the interest forecast; the terminal value is</t>
         </is>
       </c>
     </row>
@@ -2556,111 +2556,111 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>15.2%</t>
+          <t>16.9%</t>
         </is>
       </c>
       <c r="B6" s="7" t="n">
-        <v>51.75154484595317</v>
+        <v>43.96333700522357</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>53.58598972095123</v>
+        <v>45.0558316371308</v>
       </c>
       <c r="D6" s="7" t="n">
-        <v>55.71660640416448</v>
+        <v>46.27985550690241</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>58.23977514128349</v>
+        <v>47.67154681268777</v>
       </c>
       <c r="F6" s="7" t="n">
-        <v>61.29878307978106</v>
+        <v>49.28161729015513</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>16.2%</t>
+          <t>17.9%</t>
         </is>
       </c>
       <c r="B7" s="7" t="n">
-        <v>46.92330884452585</v>
+        <v>40.22564474122171</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>48.27673925934022</v>
+        <v>41.02484689888828</v>
       </c>
       <c r="D7" s="7" t="n">
-        <v>49.81551773527278</v>
+        <v>41.90108672825765</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>51.59405782760725</v>
+        <v>42.87375476913063</v>
       </c>
       <c r="F7" s="7" t="n">
-        <v>53.69038277439329</v>
+        <v>43.96934506854262</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>17.2%</t>
+          <t>18.9%</t>
         </is>
       </c>
       <c r="B8" s="7" t="n">
-        <v>42.78567612194627</v>
+        <v>36.96711651706934</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>43.7814301475257</v>
+        <v>37.54306015126826</v>
       </c>
       <c r="D8" s="7" t="n">
-        <v>44.89000036914447</v>
+        <v>38.15941321679352</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>46.14155462610511</v>
+        <v>38.82555954079371</v>
       </c>
       <c r="F8" s="7" t="n">
-        <v>47.57806945522615</v>
+        <v>39.55403218844242</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>18.2%</t>
+          <t>19.9%</t>
         </is>
       </c>
       <c r="B9" s="7" t="n">
-        <v>39.20208987342894</v>
+        <v>34.10243663491075</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>39.92793436920949</v>
+        <v>34.50664404257189</v>
       </c>
       <c r="D9" s="7" t="n">
-        <v>40.71828410658065</v>
+        <v>34.92642321660981</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>41.58897655466522</v>
+        <v>35.36513041744239</v>
       </c>
       <c r="F9" s="7" t="n">
-        <v>42.56149591582977</v>
+        <v>35.827161087566</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>19.2%</t>
+          <t>20.9%</t>
         </is>
       </c>
       <c r="B10" s="7" t="n">
-        <v>36.06968942362016</v>
+        <v>31.56534888301272</v>
       </c>
       <c r="C10" s="7" t="n">
-        <v>36.58938119058816</v>
+        <v>31.83633198870487</v>
       </c>
       <c r="D10" s="7" t="n">
-        <v>37.14100170621704</v>
+        <v>32.10598407349156</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>37.73179715426411</v>
+        <v>32.37403748526719</v>
       </c>
       <c r="F10" s="7" t="n">
-        <v>38.3713858505013</v>
+        <v>32.64014765406989</v>
       </c>
     </row>
     <row r="12">
@@ -2701,111 +2701,111 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>terminal 15.2%</t>
+          <t>terminal 16.9%</t>
         </is>
       </c>
       <c r="B14" s="7" t="n">
-        <v>65.07928889866324</v>
+        <v>52.38644918803324</v>
       </c>
       <c r="C14" s="7" t="n">
-        <v>63.15563431199472</v>
+        <v>50.80671789004094</v>
       </c>
       <c r="D14" s="7" t="n">
-        <v>61.29878307978106</v>
+        <v>49.28161729015513</v>
       </c>
       <c r="E14" s="7" t="n">
-        <v>59.50583189191774</v>
+        <v>47.80878039704058</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>57.77402971679158</v>
+        <v>46.38596407928949</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>terminal 16.2%</t>
+          <t>terminal 17.9%</t>
         </is>
       </c>
       <c r="B15" s="7" t="n">
-        <v>57.04303387246198</v>
+        <v>46.77570409711145</v>
       </c>
       <c r="C15" s="7" t="n">
-        <v>55.3371612118944</v>
+        <v>45.34789609145733</v>
       </c>
       <c r="D15" s="7" t="n">
-        <v>53.69038277439329</v>
+        <v>43.96934506854262</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>52.1001349503897</v>
+        <v>42.63792066693704</v>
       </c>
       <c r="F15" s="7" t="n">
-        <v>50.56398840677389</v>
+        <v>41.3516038526244</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>terminal 17.2%</t>
+          <t>terminal 18.9%</t>
         </is>
       </c>
       <c r="B16" s="7" t="n">
-        <v>50.58716923736989</v>
+        <v>42.1124535799006</v>
       </c>
       <c r="C16" s="7" t="n">
-        <v>49.05616591921513</v>
+        <v>40.81084521331</v>
       </c>
       <c r="D16" s="7" t="n">
-        <v>47.57806945522615</v>
+        <v>39.55403218844242</v>
       </c>
       <c r="E16" s="7" t="n">
-        <v>46.15058877372767</v>
+        <v>38.34008052530756</v>
       </c>
       <c r="F16" s="7" t="n">
-        <v>44.77155264158418</v>
+        <v>37.16715717439558</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>terminal 18.2%</t>
+          <t>terminal 19.9%</t>
         </is>
       </c>
       <c r="B17" s="7" t="n">
-        <v>45.28878322593069</v>
+        <v>38.17642784274512</v>
       </c>
       <c r="C17" s="7" t="n">
-        <v>43.90122265074462</v>
+        <v>36.98127766893269</v>
       </c>
       <c r="D17" s="7" t="n">
-        <v>42.56149591582977</v>
+        <v>35.827161087566</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>41.26753530950558</v>
+        <v>34.7123096180295</v>
       </c>
       <c r="F17" s="7" t="n">
-        <v>40.01738113023824</v>
+        <v>33.63504695170267</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>terminal 19.2%</t>
+          <t>terminal 20.9%</t>
         </is>
       </c>
       <c r="B18" s="7" t="n">
-        <v>40.86342268675902</v>
+        <v>34.81066863025118</v>
       </c>
       <c r="C18" s="7" t="n">
-        <v>39.5956036862078</v>
+        <v>33.70649786917543</v>
       </c>
       <c r="D18" s="7" t="n">
-        <v>38.3713858505013</v>
+        <v>32.64014765406989</v>
       </c>
       <c r="E18" s="7" t="n">
-        <v>37.18888774615379</v>
+        <v>31.60999079543156</v>
       </c>
       <c r="F18" s="7" t="n">
-        <v>36.04632608893751</v>
+        <v>30.61448480150225</v>
       </c>
     </row>
     <row r="20">
@@ -2840,19 +2840,19 @@
         </is>
       </c>
       <c r="B22" s="7" t="n">
-        <v>88.94087384303364</v>
+        <v>68.58093069001347</v>
       </c>
       <c r="C22" s="7" t="n">
-        <v>71.1924064433187</v>
+        <v>56.6637681487086</v>
       </c>
       <c r="D22" s="7" t="n">
-        <v>50.81803765134803</v>
+        <v>41.99307509150762</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>47.57421363061231</v>
+        <v>39.55111128728122</v>
       </c>
       <c r="F22" s="7" t="n">
-        <v>44.61511461402405</v>
+        <v>37.29653671446263</v>
       </c>
       <c r="H22" s="16">
         <f>MAX(B22:F22)-MIN(B22:F22)</f>
@@ -2866,19 +2866,19 @@
         </is>
       </c>
       <c r="B23" s="7" t="n">
-        <v>47.57806945522615</v>
+        <v>39.55403218844242</v>
       </c>
       <c r="C23" s="7" t="n">
-        <v>47.57806945522615</v>
+        <v>39.55403218844242</v>
       </c>
       <c r="D23" s="7" t="n">
-        <v>47.57806945522615</v>
+        <v>39.55403218844242</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>47.57806945522615</v>
+        <v>39.55403218844242</v>
       </c>
       <c r="F23" s="7" t="n">
-        <v>47.57806945522615</v>
+        <v>39.55403218844242</v>
       </c>
       <c r="H23" s="16">
         <f>MAX(B23:F23)-MIN(B23:F23)</f>
@@ -2892,19 +2892,19 @@
         </is>
       </c>
       <c r="B24" s="7" t="n">
-        <v>26.73474268688304</v>
+        <v>21.1572259310297</v>
       </c>
       <c r="C24" s="7" t="n">
-        <v>37.15640607105463</v>
+        <v>30.35562905973608</v>
       </c>
       <c r="D24" s="7" t="n">
-        <v>47.57806945522615</v>
+        <v>39.55403218844242</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>57.99973283939774</v>
+        <v>48.75243531714879</v>
       </c>
       <c r="F24" s="7" t="n">
-        <v>68.42139622356929</v>
+        <v>57.95083844585515</v>
       </c>
       <c r="H24" s="16">
         <f>MAX(B24:F24)-MIN(B24:F24)</f>
@@ -2918,19 +2918,19 @@
         </is>
       </c>
       <c r="B25" s="7" t="n">
-        <v>47.57806945522615</v>
+        <v>39.55403218844242</v>
       </c>
       <c r="C25" s="7" t="n">
-        <v>47.57806945522615</v>
+        <v>39.55403218844242</v>
       </c>
       <c r="D25" s="7" t="n">
-        <v>47.57806945522615</v>
+        <v>39.55403218844242</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>47.57806945522615</v>
+        <v>39.55403218844242</v>
       </c>
       <c r="F25" s="7" t="n">
-        <v>47.57806945522615</v>
+        <v>39.55403218844242</v>
       </c>
       <c r="H25" s="16">
         <f>MAX(B25:F25)-MIN(B25:F25)</f>
@@ -2944,19 +2944,19 @@
         </is>
       </c>
       <c r="B26" s="7" t="n">
-        <v>54.35297381891678</v>
+        <v>45.9728342669975</v>
       </c>
       <c r="C26" s="7" t="n">
-        <v>50.84871294114577</v>
+        <v>42.65276422636556</v>
       </c>
       <c r="D26" s="7" t="n">
-        <v>47.57806945522615</v>
+        <v>39.55403218844242</v>
       </c>
       <c r="E26" s="7" t="n">
-        <v>43.84019118560374</v>
+        <v>36.0126241451017</v>
       </c>
       <c r="F26" s="7" t="n">
-        <v>40.33593030783275</v>
+        <v>32.69255410446976</v>
       </c>
       <c r="H26" s="16">
         <f>MAX(B26:F26)-MIN(B26:F26)</f>
@@ -2970,19 +2970,19 @@
         </is>
       </c>
       <c r="B27" s="7" t="n">
-        <v>44.5245675843202</v>
+        <v>37.12797586843043</v>
       </c>
       <c r="C27" s="7" t="n">
-        <v>50.44728335978145</v>
+        <v>42.01052838980433</v>
       </c>
       <c r="D27" s="7" t="n">
-        <v>54.475229952078</v>
+        <v>45.33107618169043</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>59.55915378356799</v>
+        <v>49.52214765345646</v>
       </c>
       <c r="F27" s="7" t="n">
-        <v>62.29271491070394</v>
+        <v>51.77563343255211</v>
       </c>
       <c r="H27" s="16">
         <f>MAX(B27:F27)-MIN(B27:F27)</f>
@@ -2996,19 +2996,19 @@
         </is>
       </c>
       <c r="B28" s="7" t="n">
-        <v>42.78567612194627</v>
+        <v>36.96711651706934</v>
       </c>
       <c r="C28" s="7" t="n">
-        <v>43.7814301475257</v>
+        <v>37.54306015126826</v>
       </c>
       <c r="D28" s="7" t="n">
-        <v>44.89000036914447</v>
+        <v>38.15941321679352</v>
       </c>
       <c r="E28" s="7" t="n">
-        <v>46.14155462610511</v>
+        <v>38.82555954079371</v>
       </c>
       <c r="F28" s="7" t="n">
-        <v>47.57806945522615</v>
+        <v>39.55403218844242</v>
       </c>
       <c r="H28" s="16">
         <f>MAX(B28:F28)-MIN(B28:F28)</f>
@@ -4015,14 +4015,14 @@
         </is>
       </c>
       <c r="B5" s="7" t="n">
-        <v>18.93534675964298</v>
+        <v>15.72400503791313</v>
       </c>
       <c r="C5" s="8">
         <f>DCF!C62</f>
         <v/>
       </c>
       <c r="D5" s="7" t="n">
-        <v>85.99664201115992</v>
+        <v>71.71181857114279</v>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
@@ -4428,7 +4428,7 @@
         </is>
       </c>
       <c r="C6" s="7" t="n">
-        <v>18.93534675964298</v>
+        <v>15.72400503791313</v>
       </c>
     </row>
     <row r="7">
@@ -4443,7 +4443,7 @@
         </is>
       </c>
       <c r="C7" s="7" t="n">
-        <v>85.99664201115992</v>
+        <v>71.71181857114279</v>
       </c>
     </row>
     <row r="8">
@@ -4531,7 +4531,7 @@
       </c>
       <c r="C16" s="22" t="inlineStr">
         <is>
-          <t>28.8% → 17.2%</t>
+          <t>28.8% → 18.9%</t>
         </is>
       </c>
     </row>
@@ -4553,7 +4553,7 @@
         </is>
       </c>
       <c r="C18" s="7" t="n">
-        <v>60.92524917987439</v>
+        <v>57.0082753077468</v>
       </c>
     </row>
     <row r="19">
@@ -4634,13 +4634,13 @@
         </is>
       </c>
       <c r="C24" s="7" t="n">
-        <v>64.40329970107479</v>
+        <v>54.98853902732677</v>
       </c>
       <c r="D24" s="7" t="n">
-        <v>33.54633805623964</v>
+        <v>31.99082144464806</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>58.7640416846734</v>
+        <v>50.72202890203657</v>
       </c>
     </row>
     <row r="25">
@@ -4655,13 +4655,13 @@
         </is>
       </c>
       <c r="C25" s="7" t="n">
-        <v>50.06967725437205</v>
+        <v>41.34067083109784</v>
       </c>
       <c r="D25" s="7" t="n">
-        <v>44.9626128412424</v>
+        <v>40.07659417818311</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>60.92524917987439</v>
+        <v>57.0082753077468</v>
       </c>
     </row>
     <row r="26">
@@ -5194,7 +5194,7 @@
         </is>
       </c>
       <c r="C36" s="21" t="n">
-        <v>0.105</v>
+        <v>0.125</v>
       </c>
     </row>
     <row r="37">

</xml_diff>